<commit_message>
DVI V2: plainer headings; friendly colour-coded sheet for Milos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QvLHRX1rY5c7HuyoMWVGpU
</commit_message>
<xml_diff>
--- a/build/digital-inspections-v2/currency-2026-10-14/notify/DVI-V2-Feature-Squad_Test-cases-with-changed-behaviour_for-Viktoria-Videnovic-and-Vladimir-Tomovic_2026-10-14.xlsx
+++ b/build/digital-inspections-v2/currency-2026-10-14/notify/DVI-V2-Feature-Squad_Test-cases-with-changed-behaviour_for-Viktoria-Videnovic-and-Vladimir-Tomovic_2026-10-14.xlsx
@@ -688,12 +688,12 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Case</t>
+          <t>Test case</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Case title</t>
+          <t>Test case title</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
@@ -703,17 +703,17 @@
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>What changed in behaviour</t>
+          <t>What changed</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>What a tester sees differently (proof)</t>
+          <t>What a tester now sees differently</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>Spec rule and when the spec changed it</t>
+          <t>Where this comes from, and when it changed</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="L1" s="5" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Link to the spec</t>
         </is>
       </c>
     </row>
@@ -2306,17 +2306,17 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Why it is needed (which change)</t>
+          <t>Why it is needed (what changed)</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>Spec rule or decision, and when it changed</t>
+          <t>Where this comes from, and when it changed</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>Preconditions</t>
+          <t>Before you start</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
@@ -2326,12 +2326,12 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>Expected behaviour</t>
+          <t>What you should see</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>Next to existing case</t>
+          <t>Related existing test case</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
@@ -2876,27 +2876,27 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Possible new test</t>
+          <t>Possible new test case</t>
         </is>
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Question for product (Milos)</t>
+          <t>Question for Milos (product)</t>
         </is>
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>What the sources say today</t>
+          <t>What we know today</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>Spec rule or decision, and when</t>
+          <t>Where this comes from, and when</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>Next to existing case</t>
+          <t>Related existing test case</t>
         </is>
       </c>
     </row>

</xml_diff>